<commit_message>
feat: CIF visible en la hoja Depositos de la plantilla v1.1.0
El cliente escribe su CIF en Depositos!J2 (celda etiquetada a la vista);
la hoja Metadata lo referencia con fórmula para la lectura automática.
Confirmado: Cuentas pertenece a Banca de Empresas.
</commit_message>
<xml_diff>
--- a/docs/plantillas/CH-TPL-Depositos-v1.1.0.xlsx
+++ b/docs/plantillas/CH-TPL-Depositos-v1.1.0.xlsx
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="33">
   <si>
     <t>Depositos</t>
   </si>
@@ -151,6 +151,9 @@
   </si>
   <si>
     <t>1.0.0</t>
+  </si>
+  <si>
+    <t>CIF del Cliente:</t>
   </si>
   <si>
     <t>ClientCIF</t>
@@ -2667,6 +2670,11 @@
         <v>✔️</v>
       </c>
     </row>
+    <row r="2" spans="9:10">
+      <c r="I2" t="s">
+        <v>30</v>
+      </c>
+    </row>
     <row r="3" spans="3:23" ht="18.600000000000001" customHeight="1" thickBot="1">
       <c r="I3" s="1" t="s">
         <v>0</v>
@@ -12526,12 +12534,15 @@
         <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="B3">
+        <f>Depositos!J2</f>
       </c>
     </row>
   </sheetData>

</xml_diff>